<commit_message>
some scripts add and update
</commit_message>
<xml_diff>
--- a/_other/WeekPlan.xlsx
+++ b/_other/WeekPlan.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Dev\exchange\RichLaughter\_other\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E25F8D59-D3F6-4523-89CC-3ED5A2BA798F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F719E47B-1EB1-476F-A0A1-DEA1E5F2B676}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="163" uniqueCount="161">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="170" uniqueCount="168">
   <si>
     <t>Новый тест с использованием БД</t>
   </si>
@@ -509,6 +509,27 @@
   </si>
   <si>
     <t>PTA19_IMPERIUS</t>
+  </si>
+  <si>
+    <t>extremes_fractals</t>
+  </si>
+  <si>
+    <t>чистить дбшки через проверку наличия в wss</t>
+  </si>
+  <si>
+    <t>Индикатор зебры (%-ый ход)</t>
+  </si>
+  <si>
+    <t>Проверка исполнения таблице сделок</t>
+  </si>
+  <si>
+    <t>Изучить все индикаторы, которые сейчас есть в проекте</t>
+  </si>
+  <si>
+    <t>Создать таблицу анализа действий Qtrader. Выяснить причину лишних сделок</t>
+  </si>
+  <si>
+    <t>Дописать новые батники</t>
   </si>
 </sst>
 </file>
@@ -1015,6 +1036,12 @@
       <c r="O2" s="2" t="s">
         <v>152</v>
       </c>
+      <c r="P2" s="2" t="s">
+        <v>163</v>
+      </c>
+      <c r="Q2" s="2" t="s">
+        <v>165</v>
+      </c>
       <c r="R2" s="2" t="s">
         <v>5</v>
       </c>
@@ -1047,11 +1074,14 @@
       <c r="L3" s="4" t="s">
         <v>116</v>
       </c>
-      <c r="O3" s="2" t="s">
-        <v>127</v>
+      <c r="O3" s="12" t="s">
+        <v>166</v>
       </c>
       <c r="P3" s="2" t="s">
         <v>144</v>
+      </c>
+      <c r="Q3" s="2" t="s">
+        <v>154</v>
       </c>
       <c r="R3" s="2" t="s">
         <v>107</v>
@@ -1082,8 +1112,8 @@
       <c r="L4" s="4" t="s">
         <v>114</v>
       </c>
-      <c r="O4" s="2" t="s">
-        <v>126</v>
+      <c r="O4" s="4" t="s">
+        <v>167</v>
       </c>
       <c r="P4" s="2" t="s">
         <v>131</v>
@@ -1188,7 +1218,7 @@
         <v>132</v>
       </c>
       <c r="P7" s="2" t="s">
-        <v>139</v>
+        <v>127</v>
       </c>
       <c r="R7" s="2" t="s">
         <v>69</v>
@@ -1252,7 +1282,7 @@
         <v>141</v>
       </c>
       <c r="P9" s="2" t="s">
-        <v>154</v>
+        <v>126</v>
       </c>
       <c r="R9" s="2" t="s">
         <v>130</v>
@@ -1280,7 +1310,7 @@
       <c r="L10" s="4" t="s">
         <v>122</v>
       </c>
-      <c r="O10" s="2" t="s">
+      <c r="O10" s="4" t="s">
         <v>153</v>
       </c>
       <c r="R10" s="2" t="s">
@@ -1367,7 +1397,7 @@
       <c r="L13" s="4" t="s">
         <v>121</v>
       </c>
-      <c r="O13" s="12" t="s">
+      <c r="O13" s="4" t="s">
         <v>157</v>
       </c>
       <c r="R13" s="2" t="s">
@@ -1416,8 +1446,11 @@
       <c r="L15" s="7" t="s">
         <v>148</v>
       </c>
-    </row>
-    <row r="16" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="O15" s="7" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="16" spans="1:25" ht="30" x14ac:dyDescent="0.25">
       <c r="A16" s="2">
         <v>15</v>
       </c>
@@ -1429,6 +1462,9 @@
       </c>
       <c r="E16" s="7" t="s">
         <v>92</v>
+      </c>
+      <c r="O16" s="4" t="s">
+        <v>162</v>
       </c>
     </row>
     <row r="17" spans="1:15" ht="30" x14ac:dyDescent="0.25">
@@ -1444,8 +1480,11 @@
       <c r="E17" s="4" t="s">
         <v>93</v>
       </c>
-    </row>
-    <row r="18" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="O17" s="2" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="18" spans="1:15" ht="45" x14ac:dyDescent="0.25">
       <c r="A18" s="2">
         <v>17</v>
       </c>
@@ -1457,6 +1496,9 @@
       </c>
       <c r="E18" s="7" t="s">
         <v>94</v>
+      </c>
+      <c r="O18" s="2" t="s">
+        <v>139</v>
       </c>
     </row>
     <row r="19" spans="1:15" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
update sgs and VT5
</commit_message>
<xml_diff>
--- a/_other/WeekPlan.xlsx
+++ b/_other/WeekPlan.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Dev\exchange\RichLaughter\_other\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C3C5C295-1704-4B0A-A530-565FFF1875AA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{04D5C61B-CA0F-41CE-B8AF-584D7EDA1D65}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,17 +16,26 @@
     <sheet name="Лист1" sheetId="1" r:id="rId1"/>
     <sheet name="Идеи" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="182" uniqueCount="180">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="186" uniqueCount="184">
   <si>
     <t>Новый тест с использованием БД</t>
   </si>
@@ -520,9 +529,6 @@
     <t>Индикатор зебры (%-ый ход)</t>
   </si>
   <si>
-    <t>Проверка исполнения таблице сделок</t>
-  </si>
-  <si>
     <t>Изучить все индикаторы, которые сейчас есть в проекте</t>
   </si>
   <si>
@@ -566,6 +572,21 @@
   </si>
   <si>
     <t>Реализовать нейронку с дискретными фичами, как цель выбрать результат фейк-бота по зигзагу</t>
+  </si>
+  <si>
+    <t>Пересмотреть политику закрытия сделок VT в 18:26</t>
+  </si>
+  <si>
+    <t>Сделать разные критерии оценки Эвол. Моделей</t>
+  </si>
+  <si>
+    <t>PTA20_HANZO</t>
+  </si>
+  <si>
+    <t>PTA20_HOGGER</t>
+  </si>
+  <si>
+    <t>Добавить группы параметров к эвол. Моделям</t>
   </si>
 </sst>
 </file>
@@ -1070,10 +1091,13 @@
         <v>54</v>
       </c>
       <c r="O2" s="4" t="s">
-        <v>166</v>
+        <v>165</v>
+      </c>
+      <c r="P2" s="12" t="s">
+        <v>174</v>
       </c>
       <c r="Q2" s="2" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="R2" s="2" t="s">
         <v>5</v>
@@ -1108,7 +1132,10 @@
         <v>116</v>
       </c>
       <c r="O3" s="4" t="s">
-        <v>167</v>
+        <v>166</v>
+      </c>
+      <c r="P3" s="4" t="s">
+        <v>179</v>
       </c>
       <c r="Q3" s="2" t="s">
         <v>154</v>
@@ -1145,6 +1172,9 @@
       <c r="O4" s="4" t="s">
         <v>123</v>
       </c>
+      <c r="P4" s="9" t="s">
+        <v>175</v>
+      </c>
       <c r="Q4" s="2" t="s">
         <v>132</v>
       </c>
@@ -1177,6 +1207,9 @@
       <c r="O5" s="4" t="s">
         <v>142</v>
       </c>
+      <c r="P5" s="2" t="s">
+        <v>180</v>
+      </c>
       <c r="Q5" s="2" t="s">
         <v>140</v>
       </c>
@@ -1187,7 +1220,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="6" spans="1:25" ht="45" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:25" ht="60" x14ac:dyDescent="0.25">
       <c r="A6" s="2">
         <v>5</v>
       </c>
@@ -1212,6 +1245,9 @@
       <c r="O6" s="4" t="s">
         <v>153</v>
       </c>
+      <c r="P6" s="4" t="s">
+        <v>152</v>
+      </c>
       <c r="Q6" s="2" t="s">
         <v>141</v>
       </c>
@@ -1222,7 +1258,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="7" spans="1:25" ht="60" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:25" ht="45" x14ac:dyDescent="0.25">
       <c r="A7" s="2">
         <v>6</v>
       </c>
@@ -1247,8 +1283,11 @@
       <c r="O7" s="4" t="s">
         <v>157</v>
       </c>
+      <c r="P7" s="2" t="s">
+        <v>183</v>
+      </c>
       <c r="Q7" s="2" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="R7" s="2" t="s">
         <v>69</v>
@@ -1277,10 +1316,10 @@
         <v>118</v>
       </c>
       <c r="O8" s="4" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="Q8" s="2" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="R8" s="2" t="s">
         <v>70</v>
@@ -1312,7 +1351,7 @@
         <v>161</v>
       </c>
       <c r="Q9" s="2" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="R9" s="2" t="s">
         <v>130</v>
@@ -1321,7 +1360,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="10" spans="1:25" ht="30" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:25" ht="45" x14ac:dyDescent="0.25">
       <c r="A10" s="2">
         <v>9</v>
       </c>
@@ -1344,7 +1383,7 @@
         <v>162</v>
       </c>
       <c r="Q10" s="2" t="s">
-        <v>158</v>
+        <v>139</v>
       </c>
       <c r="R10" s="2" t="s">
         <v>133</v>
@@ -1372,11 +1411,11 @@
       <c r="L11" s="4" t="s">
         <v>124</v>
       </c>
-      <c r="O11" s="2" t="s">
-        <v>175</v>
+      <c r="O11" s="4" t="s">
+        <v>168</v>
       </c>
       <c r="Q11" s="2" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="R11" s="2" t="s">
         <v>134</v>
@@ -1385,7 +1424,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="12" spans="1:25" ht="45" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:25" ht="90" x14ac:dyDescent="0.25">
       <c r="A12" s="2">
         <v>11</v>
       </c>
@@ -1404,11 +1443,11 @@
       <c r="L12" s="4" t="s">
         <v>125</v>
       </c>
-      <c r="O12" s="12" t="s">
-        <v>176</v>
+      <c r="O12" s="4" t="s">
+        <v>145</v>
       </c>
       <c r="Q12" s="2" t="s">
-        <v>139</v>
+        <v>144</v>
       </c>
       <c r="R12" s="2" t="s">
         <v>135</v>
@@ -1417,7 +1456,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="13" spans="1:25" ht="60" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:25" ht="45" x14ac:dyDescent="0.25">
       <c r="A13" s="2">
         <v>12</v>
       </c>
@@ -1436,20 +1475,20 @@
       <c r="L13" s="4" t="s">
         <v>121</v>
       </c>
-      <c r="O13" s="12" t="s">
-        <v>179</v>
+      <c r="O13" s="7" t="s">
+        <v>146</v>
       </c>
       <c r="Q13" s="2" t="s">
-        <v>163</v>
+        <v>131</v>
       </c>
       <c r="R13" s="2" t="s">
         <v>136</v>
       </c>
       <c r="S13" s="9" t="s">
-        <v>172</v>
-      </c>
-    </row>
-    <row r="14" spans="1:25" ht="90" x14ac:dyDescent="0.25">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="14" spans="1:25" ht="60" x14ac:dyDescent="0.25">
       <c r="A14" s="2">
         <v>13</v>
       </c>
@@ -1468,11 +1507,17 @@
       <c r="L14" s="4" t="s">
         <v>147</v>
       </c>
+      <c r="O14" s="7" t="s">
+        <v>159</v>
+      </c>
       <c r="Q14" s="2" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="15" spans="1:25" x14ac:dyDescent="0.25">
+        <v>137</v>
+      </c>
+      <c r="R14" s="9" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="15" spans="1:25" ht="30" x14ac:dyDescent="0.25">
       <c r="A15" s="2">
         <v>14</v>
       </c>
@@ -1491,11 +1536,14 @@
       <c r="L15" s="7" t="s">
         <v>148</v>
       </c>
+      <c r="O15" s="7" t="s">
+        <v>160</v>
+      </c>
       <c r="Q15" s="2" t="s">
-        <v>131</v>
-      </c>
-    </row>
-    <row r="16" spans="1:25" ht="60" x14ac:dyDescent="0.25">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="16" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A16" s="2">
         <v>15</v>
       </c>
@@ -1508,8 +1556,14 @@
       <c r="E16" s="7" t="s">
         <v>92</v>
       </c>
+      <c r="O16" s="4" t="s">
+        <v>169</v>
+      </c>
+      <c r="P16" s="4" t="s">
+        <v>181</v>
+      </c>
       <c r="Q16" s="2" t="s">
-        <v>137</v>
+        <v>127</v>
       </c>
     </row>
     <row r="17" spans="1:17" ht="30" x14ac:dyDescent="0.25">
@@ -1525,8 +1579,14 @@
       <c r="E17" s="4" t="s">
         <v>93</v>
       </c>
+      <c r="O17" s="7" t="s">
+        <v>172</v>
+      </c>
+      <c r="P17" s="7" t="s">
+        <v>182</v>
+      </c>
       <c r="Q17" s="2" t="s">
-        <v>138</v>
+        <v>120</v>
       </c>
     </row>
     <row r="18" spans="1:17" x14ac:dyDescent="0.25">
@@ -1542,11 +1602,14 @@
       <c r="E18" s="7" t="s">
         <v>94</v>
       </c>
+      <c r="O18" s="7" t="s">
+        <v>173</v>
+      </c>
       <c r="Q18" s="2" t="s">
-        <v>127</v>
-      </c>
-    </row>
-    <row r="19" spans="1:17" x14ac:dyDescent="0.25">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="19" spans="1:17" ht="30" x14ac:dyDescent="0.25">
       <c r="A19" s="2">
         <v>18</v>
       </c>
@@ -1560,13 +1623,13 @@
         <v>95</v>
       </c>
       <c r="O19" s="4" t="s">
-        <v>169</v>
+        <v>177</v>
       </c>
       <c r="Q19" s="2" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="20" spans="1:17" x14ac:dyDescent="0.25">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="20" spans="1:17" ht="45" x14ac:dyDescent="0.25">
       <c r="A20" s="2">
         <v>19</v>
       </c>
@@ -1579,14 +1642,11 @@
       <c r="E20" s="7" t="s">
         <v>96</v>
       </c>
-      <c r="O20" s="4" t="s">
-        <v>145</v>
-      </c>
       <c r="Q20" s="2" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="21" spans="1:17" ht="30" x14ac:dyDescent="0.25">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="21" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A21" s="2">
         <v>20</v>
       </c>
@@ -1596,14 +1656,8 @@
       <c r="E21" s="4" t="s">
         <v>97</v>
       </c>
-      <c r="O21" s="7" t="s">
-        <v>146</v>
-      </c>
-      <c r="Q21" s="2" t="s">
-        <v>168</v>
-      </c>
-    </row>
-    <row r="22" spans="1:17" ht="45" x14ac:dyDescent="0.25">
+    </row>
+    <row r="22" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A22" s="2">
         <v>21</v>
       </c>
@@ -1612,12 +1666,6 @@
       </c>
       <c r="E22" s="7" t="s">
         <v>98</v>
-      </c>
-      <c r="O22" s="7" t="s">
-        <v>159</v>
-      </c>
-      <c r="Q22" s="2" t="s">
-        <v>171</v>
       </c>
     </row>
     <row r="23" spans="1:17" x14ac:dyDescent="0.25">
@@ -1630,9 +1678,6 @@
       <c r="E23" s="7" t="s">
         <v>99</v>
       </c>
-      <c r="O23" s="7" t="s">
-        <v>160</v>
-      </c>
     </row>
     <row r="24" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A24" s="2">
@@ -1644,9 +1689,6 @@
       <c r="E24" s="7" t="s">
         <v>100</v>
       </c>
-      <c r="O24" s="4" t="s">
-        <v>170</v>
-      </c>
     </row>
     <row r="25" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A25" s="2">
@@ -1658,9 +1700,6 @@
       <c r="E25" s="7" t="s">
         <v>101</v>
       </c>
-      <c r="O25" s="7" t="s">
-        <v>173</v>
-      </c>
     </row>
     <row r="26" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A26" s="2">
@@ -1672,9 +1711,6 @@
       <c r="E26" s="7" t="s">
         <v>102</v>
       </c>
-      <c r="O26" s="7" t="s">
-        <v>174</v>
-      </c>
     </row>
     <row r="27" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A27" s="2">
@@ -1682,9 +1718,6 @@
       </c>
       <c r="D27" s="7" t="s">
         <v>62</v>
-      </c>
-      <c r="O27" s="4" t="s">
-        <v>178</v>
       </c>
     </row>
     <row r="28" spans="1:17" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
update analys_dbs and add PTA21_WHITEMANE
</commit_message>
<xml_diff>
--- a/_other/WeekPlan.xlsx
+++ b/_other/WeekPlan.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Dev\exchange\RichLaughter\_other\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{32612D24-5BF9-4786-A08D-98EBEBB1D13F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1F0EDA0A-63E9-4143-BDA3-95EED4EE7609}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="193" uniqueCount="191">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="195" uniqueCount="193">
   <si>
     <t>Новый тест с использованием БД</t>
   </si>
@@ -430,9 +430,6 @@
     <t>Робот на percent_zigzag</t>
   </si>
   <si>
-    <t>Робот по 4 точкам зигзага (выбрасываем последнюю)</t>
-  </si>
-  <si>
     <t>Канал допуска относительно удаленности от СС</t>
   </si>
   <si>
@@ -608,6 +605,15 @@
   </si>
   <si>
     <t>Вывод графиков с fee при оптимизации</t>
+  </si>
+  <si>
+    <t>Робот с паттернами VSA</t>
+  </si>
+  <si>
+    <t>Новый тестер стратегий</t>
+  </si>
+  <si>
+    <t>Среднедневная прибыль для analys_dbs</t>
   </si>
 </sst>
 </file>
@@ -1103,13 +1109,13 @@
         <v>54</v>
       </c>
       <c r="O2" s="4" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="P2" s="4" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="Q2" s="2" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="R2" s="2" t="s">
         <v>5</v>
@@ -1144,13 +1150,13 @@
         <v>116</v>
       </c>
       <c r="O3" s="4" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="P3" s="4" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="Q3" s="2" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="R3" s="2" t="s">
         <v>107</v>
@@ -1185,10 +1191,10 @@
         <v>123</v>
       </c>
       <c r="P4" s="9" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="Q4" s="2" t="s">
-        <v>131</v>
+        <v>138</v>
       </c>
       <c r="R4" s="2" t="s">
         <v>106</v>
@@ -1217,10 +1223,10 @@
         <v>115</v>
       </c>
       <c r="O5" s="4" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="P5" s="2" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="Q5" s="2" t="s">
         <v>139</v>
@@ -1229,7 +1235,7 @@
         <v>51</v>
       </c>
       <c r="S5" s="2" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
     </row>
     <row r="6" spans="1:25" ht="60" x14ac:dyDescent="0.25">
@@ -1255,13 +1261,13 @@
         <v>110</v>
       </c>
       <c r="O6" s="4" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="P6" s="4" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="Q6" s="2" t="s">
-        <v>140</v>
+        <v>153</v>
       </c>
       <c r="R6" s="2" t="s">
         <v>76</v>
@@ -1293,10 +1299,10 @@
         <v>117</v>
       </c>
       <c r="O7" s="4" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="P7" s="2" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="Q7" s="2" t="s">
         <v>154</v>
@@ -1328,13 +1334,13 @@
         <v>118</v>
       </c>
       <c r="O8" s="4" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="P8" s="4" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="Q8" s="2" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="R8" s="2" t="s">
         <v>70</v>
@@ -1343,7 +1349,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="9" spans="1:25" ht="45" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:25" ht="90" x14ac:dyDescent="0.25">
       <c r="A9" s="2">
         <v>8</v>
       </c>
@@ -1363,13 +1369,13 @@
         <v>119</v>
       </c>
       <c r="O9" s="7" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="P9" s="4" t="s">
         <v>120</v>
       </c>
       <c r="Q9" s="2" t="s">
-        <v>157</v>
+        <v>142</v>
       </c>
       <c r="R9" s="2" t="s">
         <v>129</v>
@@ -1378,7 +1384,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="10" spans="1:25" ht="90" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:25" ht="45" x14ac:dyDescent="0.25">
       <c r="A10" s="2">
         <v>9</v>
       </c>
@@ -1398,16 +1404,16 @@
         <v>122</v>
       </c>
       <c r="O10" s="4" t="s">
-        <v>161</v>
-      </c>
-      <c r="P10" s="2" t="s">
-        <v>138</v>
+        <v>160</v>
+      </c>
+      <c r="P10" s="4" t="s">
+        <v>137</v>
       </c>
       <c r="Q10" s="2" t="s">
-        <v>143</v>
+        <v>130</v>
       </c>
       <c r="R10" s="2" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="S10" s="2" t="s">
         <v>38</v>
@@ -1433,22 +1439,22 @@
         <v>124</v>
       </c>
       <c r="O11" s="4" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="P11" s="2" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="Q11" s="2" t="s">
-        <v>130</v>
+        <v>135</v>
       </c>
       <c r="R11" s="2" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="S11" s="2" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="12" spans="1:25" ht="60" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:25" ht="45" x14ac:dyDescent="0.25">
       <c r="A12" s="2">
         <v>11</v>
       </c>
@@ -1468,16 +1474,16 @@
         <v>125</v>
       </c>
       <c r="O12" s="4" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="P12" s="2" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="Q12" s="2" t="s">
         <v>136</v>
       </c>
       <c r="R12" s="2" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="S12" s="2" t="s">
         <v>78</v>
@@ -1503,19 +1509,19 @@
         <v>121</v>
       </c>
       <c r="O13" s="7" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="P13" s="2" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="Q13" s="2" t="s">
-        <v>137</v>
+        <v>126</v>
       </c>
       <c r="R13" s="2" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="S13" s="9" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
     </row>
     <row r="14" spans="1:25" ht="60" x14ac:dyDescent="0.25">
@@ -1535,19 +1541,22 @@
         <v>89</v>
       </c>
       <c r="L14" s="4" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="O14" s="7" t="s">
-        <v>158</v>
+        <v>157</v>
+      </c>
+      <c r="P14" s="2" t="s">
+        <v>191</v>
       </c>
       <c r="Q14" s="2" t="s">
-        <v>126</v>
+        <v>165</v>
       </c>
       <c r="R14" s="9" t="s">
-        <v>177</v>
-      </c>
-    </row>
-    <row r="15" spans="1:25" ht="30" x14ac:dyDescent="0.25">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="15" spans="1:25" ht="45" x14ac:dyDescent="0.25">
       <c r="A15" s="2">
         <v>14</v>
       </c>
@@ -1564,19 +1573,22 @@
         <v>90</v>
       </c>
       <c r="L15" s="7" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="O15" s="7" t="s">
-        <v>159</v>
+        <v>158</v>
+      </c>
+      <c r="P15" s="4" t="s">
+        <v>192</v>
       </c>
       <c r="Q15" s="2" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="R15" s="2" t="s">
-        <v>185</v>
-      </c>
-    </row>
-    <row r="16" spans="1:25" ht="45" x14ac:dyDescent="0.25">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="16" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A16" s="2">
         <v>15</v>
       </c>
@@ -1590,13 +1602,13 @@
         <v>92</v>
       </c>
       <c r="O16" s="4" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="P16" s="4" t="s">
-        <v>180</v>
-      </c>
-      <c r="Q16" s="2" t="s">
-        <v>169</v>
+        <v>179</v>
+      </c>
+      <c r="R16" s="2" t="s">
+        <v>190</v>
       </c>
     </row>
     <row r="17" spans="1:16" ht="30" x14ac:dyDescent="0.25">
@@ -1613,10 +1625,10 @@
         <v>93</v>
       </c>
       <c r="O17" s="7" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="P17" s="7" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
     </row>
     <row r="18" spans="1:16" x14ac:dyDescent="0.25">
@@ -1633,10 +1645,10 @@
         <v>94</v>
       </c>
       <c r="O18" s="7" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="P18" s="4" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
     </row>
     <row r="19" spans="1:16" x14ac:dyDescent="0.25">
@@ -1653,10 +1665,10 @@
         <v>95</v>
       </c>
       <c r="O19" s="4" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="P19" s="7" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
     </row>
     <row r="20" spans="1:16" x14ac:dyDescent="0.25">
@@ -1673,7 +1685,7 @@
         <v>96</v>
       </c>
       <c r="P20" s="7" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
     </row>
     <row r="21" spans="1:16" x14ac:dyDescent="0.25">
@@ -1687,7 +1699,7 @@
         <v>97</v>
       </c>
       <c r="P21" s="7" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
     </row>
     <row r="22" spans="1:16" x14ac:dyDescent="0.25">
@@ -1909,7 +1921,7 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B1" s="10" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
     </row>
     <row r="2" spans="1:3" ht="90" x14ac:dyDescent="0.25">
@@ -1917,10 +1929,10 @@
         <v>1</v>
       </c>
       <c r="B2" s="10" t="s">
+        <v>148</v>
+      </c>
+      <c r="C2" s="10" t="s">
         <v>149</v>
-      </c>
-      <c r="C2" s="10" t="s">
-        <v>150</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
add checking wss step
</commit_message>
<xml_diff>
--- a/_other/WeekPlan.xlsx
+++ b/_other/WeekPlan.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Dev\exchange\RichLaughter\_other\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{492BFB2F-B0AF-4C93-80DB-2EB6F28FC893}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{45A7A1EF-7034-4808-8410-DBC079CD1D51}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="216" uniqueCount="214">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="218" uniqueCount="216">
   <si>
     <t>Новый тест с использованием БД</t>
   </si>
@@ -445,9 +445,6 @@
     <t>Фибо по зигзагу</t>
   </si>
   <si>
-    <t>Тиковый тестер</t>
-  </si>
-  <si>
     <t>pta14_ranger (определять боковик по большому adx)</t>
   </si>
   <si>
@@ -677,6 +674,15 @@
   </si>
   <si>
     <t>Разобраться с ошибкой в VT</t>
+  </si>
+  <si>
+    <t>Шаговый тестер</t>
+  </si>
+  <si>
+    <t>Протестировать все wss на шаговом тестере</t>
+  </si>
+  <si>
+    <t>PTA22_BERSERK</t>
   </si>
 </sst>
 </file>
@@ -692,7 +698,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -729,6 +735,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -742,7 +754,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -776,6 +788,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1172,13 +1187,13 @@
         <v>52</v>
       </c>
       <c r="O2" s="4" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="P2" s="4" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="Q2" s="4" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="R2" s="2" t="s">
         <v>5</v>
@@ -1187,7 +1202,7 @@
         <v>36</v>
       </c>
       <c r="T2" s="2" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
     </row>
     <row r="3" spans="1:25" ht="60" x14ac:dyDescent="0.25">
@@ -1216,22 +1231,22 @@
         <v>113</v>
       </c>
       <c r="O3" s="4" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="P3" s="4" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="Q3" s="4" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="R3" s="2" t="s">
         <v>104</v>
       </c>
       <c r="S3" s="2" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="T3" s="2" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="4" spans="1:25" ht="30" x14ac:dyDescent="0.25">
@@ -1260,10 +1275,10 @@
         <v>120</v>
       </c>
       <c r="P4" s="4" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="Q4" s="4" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="R4" s="2" t="s">
         <v>103</v>
@@ -1292,13 +1307,13 @@
         <v>112</v>
       </c>
       <c r="O5" s="4" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="P5" s="4" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="Q5" s="4" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="R5" s="2" t="s">
         <v>49</v>
@@ -1307,7 +1322,7 @@
         <v>125</v>
       </c>
       <c r="U5" s="2" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
     </row>
     <row r="6" spans="1:25" ht="45" x14ac:dyDescent="0.25">
@@ -1333,13 +1348,13 @@
         <v>107</v>
       </c>
       <c r="O6" s="4" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="P6" s="4" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="Q6" s="4" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="R6" s="2" t="s">
         <v>73</v>
@@ -1348,7 +1363,7 @@
         <v>43</v>
       </c>
       <c r="T6" s="2" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="U6" s="2" t="s">
         <v>135</v>
@@ -1377,13 +1392,13 @@
         <v>114</v>
       </c>
       <c r="O7" s="4" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="P7" s="4" t="s">
         <v>117</v>
       </c>
       <c r="Q7" s="4" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="R7" s="2" t="s">
         <v>67</v>
@@ -1392,10 +1407,10 @@
         <v>45</v>
       </c>
       <c r="T7" s="2" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="U7" s="2" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
     </row>
     <row r="8" spans="1:25" ht="90" x14ac:dyDescent="0.25">
@@ -1418,13 +1433,13 @@
         <v>115</v>
       </c>
       <c r="O8" s="4" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="P8" s="4" t="s">
         <v>134</v>
       </c>
-      <c r="Q8" s="2" t="s">
-        <v>213</v>
+      <c r="Q8" s="4" t="s">
+        <v>212</v>
       </c>
       <c r="R8" s="2" t="s">
         <v>126</v>
@@ -1433,10 +1448,10 @@
         <v>38</v>
       </c>
       <c r="T8" s="2" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="U8" s="2" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
     </row>
     <row r="9" spans="1:25" ht="60" x14ac:dyDescent="0.25">
@@ -1459,13 +1474,13 @@
         <v>116</v>
       </c>
       <c r="O9" s="4" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="P9" s="4" t="s">
-        <v>169</v>
-      </c>
-      <c r="Q9" s="2" t="s">
-        <v>136</v>
+        <v>168</v>
+      </c>
+      <c r="Q9" s="4" t="s">
+        <v>213</v>
       </c>
       <c r="R9" s="2" t="s">
         <v>128</v>
@@ -1477,7 +1492,7 @@
         <v>127</v>
       </c>
       <c r="U9" s="2" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
     </row>
     <row r="10" spans="1:25" ht="60" x14ac:dyDescent="0.25">
@@ -1500,10 +1515,13 @@
         <v>119</v>
       </c>
       <c r="O10" s="4" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="P10" s="4" t="s">
-        <v>195</v>
+        <v>194</v>
+      </c>
+      <c r="Q10" s="12" t="s">
+        <v>214</v>
       </c>
       <c r="R10" s="2" t="s">
         <v>129</v>
@@ -1515,7 +1533,7 @@
         <v>132</v>
       </c>
       <c r="U10" s="2" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
     </row>
     <row r="11" spans="1:25" ht="45" x14ac:dyDescent="0.25">
@@ -1538,10 +1556,10 @@
         <v>121</v>
       </c>
       <c r="O11" s="4" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="P11" s="4" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="R11" s="2" t="s">
         <v>130</v>
@@ -1550,7 +1568,7 @@
         <v>133</v>
       </c>
       <c r="U11" s="2" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
     </row>
     <row r="12" spans="1:25" ht="45" x14ac:dyDescent="0.25">
@@ -1573,22 +1591,22 @@
         <v>122</v>
       </c>
       <c r="O12" s="4" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="P12" s="4" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="R12" s="2" t="s">
         <v>131</v>
       </c>
       <c r="S12" s="2" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="T12" s="2" t="s">
         <v>123</v>
       </c>
       <c r="U12" s="2" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
     </row>
     <row r="13" spans="1:25" ht="60" x14ac:dyDescent="0.25">
@@ -1611,19 +1629,19 @@
         <v>118</v>
       </c>
       <c r="O13" s="4" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="P13" s="4" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="R13" s="9" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="S13" s="2" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="T13" s="2" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
     </row>
     <row r="14" spans="1:25" ht="30" x14ac:dyDescent="0.25">
@@ -1643,19 +1661,19 @@
         <v>86</v>
       </c>
       <c r="L14" s="4" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="O14" s="7" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="P14" s="4" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="S14" s="2" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="T14" s="2" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
     </row>
     <row r="15" spans="1:25" ht="30" x14ac:dyDescent="0.25">
@@ -1675,19 +1693,19 @@
         <v>87</v>
       </c>
       <c r="L15" s="7" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="O15" s="7" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="P15" s="4" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="R15" s="2" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="T15" s="2" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
     </row>
     <row r="16" spans="1:25" ht="45" x14ac:dyDescent="0.25">
@@ -1704,16 +1722,16 @@
         <v>89</v>
       </c>
       <c r="O16" s="7" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="P16" s="4" t="s">
+        <v>184</v>
+      </c>
+      <c r="R16" s="2" t="s">
         <v>185</v>
       </c>
-      <c r="R16" s="2" t="s">
-        <v>186</v>
-      </c>
       <c r="T16" s="2" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
     </row>
     <row r="17" spans="1:20" ht="45" x14ac:dyDescent="0.25">
@@ -1730,16 +1748,16 @@
         <v>90</v>
       </c>
       <c r="O17" s="4" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="P17" s="4" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="R17" s="2" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="T17" s="2" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
     </row>
     <row r="18" spans="1:20" x14ac:dyDescent="0.25">
@@ -1756,10 +1774,13 @@
         <v>91</v>
       </c>
       <c r="O18" s="7" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="P18" s="4" t="s">
-        <v>175</v>
+        <v>174</v>
+      </c>
+      <c r="Q18" s="4" t="s">
+        <v>215</v>
       </c>
     </row>
     <row r="19" spans="1:20" x14ac:dyDescent="0.25">
@@ -1776,10 +1797,10 @@
         <v>92</v>
       </c>
       <c r="O19" s="7" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="P19" s="7" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
     </row>
     <row r="20" spans="1:20" x14ac:dyDescent="0.25">
@@ -1796,10 +1817,10 @@
         <v>93</v>
       </c>
       <c r="O20" s="4" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="P20" s="4" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
     </row>
     <row r="21" spans="1:20" x14ac:dyDescent="0.25">
@@ -1813,7 +1834,7 @@
         <v>94</v>
       </c>
       <c r="P21" s="7" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
     </row>
     <row r="22" spans="1:20" x14ac:dyDescent="0.25">
@@ -1827,7 +1848,7 @@
         <v>95</v>
       </c>
       <c r="P22" s="7" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
     </row>
     <row r="23" spans="1:20" x14ac:dyDescent="0.25">
@@ -1841,7 +1862,7 @@
         <v>96</v>
       </c>
       <c r="P23" s="7" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
     </row>
     <row r="24" spans="1:20" x14ac:dyDescent="0.25">
@@ -1855,7 +1876,7 @@
         <v>97</v>
       </c>
       <c r="P24" s="4" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
     </row>
     <row r="25" spans="1:20" x14ac:dyDescent="0.25">
@@ -1869,7 +1890,7 @@
         <v>98</v>
       </c>
       <c r="P25" s="7" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
     </row>
     <row r="26" spans="1:20" x14ac:dyDescent="0.25">
@@ -2047,7 +2068,7 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B1" s="10" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
     </row>
     <row r="2" spans="1:3" ht="90" x14ac:dyDescent="0.25">
@@ -2055,10 +2076,10 @@
         <v>1</v>
       </c>
       <c r="B2" s="10" t="s">
+        <v>144</v>
+      </c>
+      <c r="C2" s="10" t="s">
         <v>145</v>
-      </c>
-      <c r="C2" s="10" t="s">
-        <v>146</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
some new ws OGTA,PSTA,STAML
</commit_message>
<xml_diff>
--- a/_other/WeekPlan.xlsx
+++ b/_other/WeekPlan.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Dev\exchange\RichLaughter\_other\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DF03999E-A0E0-4BA3-95B9-05D687122452}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1341A82E-FD0D-485C-B592-35F529497800}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="212" uniqueCount="210">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="219" uniqueCount="217">
   <si>
     <t>Новый тест с использованием БД</t>
   </si>
@@ -580,9 +580,6 @@
     <t>PTA21_AURIEL</t>
   </si>
   <si>
-    <t>Улучшить wizard</t>
-  </si>
-  <si>
     <t>Идеи для инструментов с узкими боковиками</t>
   </si>
   <si>
@@ -665,6 +662,30 @@
   </si>
   <si>
     <t>Проанализировать результаты стептеста акции</t>
+  </si>
+  <si>
+    <t>Сети КАН</t>
+  </si>
+  <si>
+    <t>OGTA4_HAMSTER</t>
+  </si>
+  <si>
+    <t>OGTA4_RAT</t>
+  </si>
+  <si>
+    <t>OGTA6_CERBERUS</t>
+  </si>
+  <si>
+    <t>OGTA7_PARADOX</t>
+  </si>
+  <si>
+    <t>Индикатор идеальной стратегии</t>
+  </si>
+  <si>
+    <t>PSTA3_REVAN</t>
+  </si>
+  <si>
+    <t>STAML2a_PHENOMENON</t>
   </si>
 </sst>
 </file>
@@ -1166,10 +1187,10 @@
         <v>159</v>
       </c>
       <c r="Q2" s="4" t="s">
-        <v>188</v>
-      </c>
-      <c r="R2" s="2" t="s">
-        <v>5</v>
+        <v>187</v>
+      </c>
+      <c r="R2" s="4" t="s">
+        <v>185</v>
       </c>
       <c r="S2" s="2" t="s">
         <v>35</v>
@@ -1177,8 +1198,11 @@
       <c r="T2" s="2" t="s">
         <v>150</v>
       </c>
-      <c r="U2" s="2" t="s">
-        <v>181</v>
+      <c r="U2" s="9" t="s">
+        <v>127</v>
+      </c>
+      <c r="V2" s="2" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="3" spans="1:25" ht="60" x14ac:dyDescent="0.25">
@@ -1213,10 +1237,10 @@
         <v>164</v>
       </c>
       <c r="Q3" s="4" t="s">
-        <v>185</v>
-      </c>
-      <c r="R3" s="2" t="s">
-        <v>98</v>
+        <v>184</v>
+      </c>
+      <c r="R3" s="4" t="s">
+        <v>214</v>
       </c>
       <c r="S3" s="2" t="s">
         <v>129</v>
@@ -1225,10 +1249,13 @@
         <v>140</v>
       </c>
       <c r="U3" s="2" t="s">
-        <v>127</v>
-      </c>
-    </row>
-    <row r="4" spans="1:25" ht="30" x14ac:dyDescent="0.25">
+        <v>149</v>
+      </c>
+      <c r="V3" s="2" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="4" spans="1:25" ht="90" x14ac:dyDescent="0.25">
       <c r="A4" s="2">
         <v>3</v>
       </c>
@@ -1257,10 +1284,7 @@
         <v>179</v>
       </c>
       <c r="Q4" s="4" t="s">
-        <v>192</v>
-      </c>
-      <c r="R4" s="2" t="s">
-        <v>69</v>
+        <v>191</v>
       </c>
       <c r="S4" s="2" t="s">
         <v>118</v>
@@ -1269,10 +1293,13 @@
         <v>141</v>
       </c>
       <c r="U4" s="2" t="s">
-        <v>149</v>
-      </c>
-    </row>
-    <row r="5" spans="1:25" ht="90" x14ac:dyDescent="0.25">
+        <v>130</v>
+      </c>
+      <c r="V4" s="2" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="5" spans="1:25" ht="60" x14ac:dyDescent="0.25">
       <c r="A5" s="2">
         <v>4</v>
       </c>
@@ -1298,10 +1325,7 @@
         <v>138</v>
       </c>
       <c r="Q5" s="4" t="s">
-        <v>196</v>
-      </c>
-      <c r="R5" s="2" t="s">
-        <v>63</v>
+        <v>195</v>
       </c>
       <c r="S5" s="2" t="s">
         <v>41</v>
@@ -1310,10 +1334,13 @@
         <v>142</v>
       </c>
       <c r="U5" s="2" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="6" spans="1:25" ht="60" x14ac:dyDescent="0.25">
+        <v>192</v>
+      </c>
+      <c r="V5" s="2" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="6" spans="1:25" ht="45" x14ac:dyDescent="0.25">
       <c r="A6" s="2">
         <v>5</v>
       </c>
@@ -1342,10 +1369,7 @@
         <v>167</v>
       </c>
       <c r="Q6" s="4" t="s">
-        <v>199</v>
-      </c>
-      <c r="R6" s="2" t="s">
-        <v>119</v>
+        <v>198</v>
       </c>
       <c r="S6" s="2" t="s">
         <v>168</v>
@@ -1355,6 +1379,9 @@
       </c>
       <c r="U6" s="2" t="s">
         <v>193</v>
+      </c>
+      <c r="V6" s="2" t="s">
+        <v>119</v>
       </c>
     </row>
     <row r="7" spans="1:25" ht="45" x14ac:dyDescent="0.25">
@@ -1386,19 +1413,19 @@
         <v>111</v>
       </c>
       <c r="Q7" s="4" t="s">
-        <v>200</v>
-      </c>
-      <c r="R7" s="2" t="s">
-        <v>121</v>
+        <v>199</v>
       </c>
       <c r="S7" s="2" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="T7" s="2" t="s">
         <v>120</v>
       </c>
       <c r="U7" s="2" t="s">
-        <v>194</v>
+        <v>209</v>
+      </c>
+      <c r="V7" s="2" t="s">
+        <v>121</v>
       </c>
     </row>
     <row r="8" spans="1:25" ht="60" x14ac:dyDescent="0.25">
@@ -1427,16 +1454,19 @@
         <v>126</v>
       </c>
       <c r="Q8" s="4" t="s">
-        <v>201</v>
-      </c>
-      <c r="R8" s="2" t="s">
-        <v>122</v>
+        <v>200</v>
       </c>
       <c r="S8" s="2" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="T8" s="2" t="s">
         <v>124</v>
+      </c>
+      <c r="U8" s="9" t="s">
+        <v>125</v>
+      </c>
+      <c r="V8" s="2" t="s">
+        <v>122</v>
       </c>
     </row>
     <row r="9" spans="1:25" ht="30" x14ac:dyDescent="0.25">
@@ -1465,16 +1495,13 @@
         <v>160</v>
       </c>
       <c r="Q9" s="4" t="s">
-        <v>202</v>
-      </c>
-      <c r="R9" s="2" t="s">
+        <v>201</v>
+      </c>
+      <c r="S9" s="2" t="s">
+        <v>204</v>
+      </c>
+      <c r="V9" s="2" t="s">
         <v>123</v>
-      </c>
-      <c r="S9" s="2" t="s">
-        <v>205</v>
-      </c>
-      <c r="T9" s="2" t="s">
-        <v>125</v>
       </c>
     </row>
     <row r="10" spans="1:25" ht="60" x14ac:dyDescent="0.25">
@@ -1500,19 +1527,19 @@
         <v>148</v>
       </c>
       <c r="P10" s="4" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="Q10" s="4" t="s">
-        <v>203</v>
-      </c>
-      <c r="R10" s="9" t="s">
-        <v>163</v>
+        <v>202</v>
       </c>
       <c r="S10" s="2" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="T10" s="2" t="s">
         <v>117</v>
+      </c>
+      <c r="V10" s="9" t="s">
+        <v>163</v>
       </c>
     </row>
     <row r="11" spans="1:25" ht="45" x14ac:dyDescent="0.25">
@@ -1540,17 +1567,17 @@
       <c r="P11" s="4" t="s">
         <v>177</v>
       </c>
-      <c r="Q11" s="2" t="s">
-        <v>195</v>
-      </c>
-      <c r="R11" s="2" t="s">
+      <c r="Q11" s="4" t="s">
+        <v>194</v>
+      </c>
+      <c r="S11" s="2" t="s">
+        <v>206</v>
+      </c>
+      <c r="T11" s="2" t="s">
+        <v>181</v>
+      </c>
+      <c r="V11" s="2" t="s">
         <v>169</v>
-      </c>
-      <c r="S11" s="2" t="s">
-        <v>207</v>
-      </c>
-      <c r="T11" s="2" t="s">
-        <v>182</v>
       </c>
     </row>
     <row r="12" spans="1:25" ht="45" x14ac:dyDescent="0.25">
@@ -1579,13 +1606,10 @@
         <v>156</v>
       </c>
       <c r="Q12" s="4" t="s">
-        <v>183</v>
-      </c>
-      <c r="R12" s="2" t="s">
+        <v>182</v>
+      </c>
+      <c r="V12" s="2" t="s">
         <v>175</v>
-      </c>
-      <c r="T12" s="2" t="s">
-        <v>186</v>
       </c>
     </row>
     <row r="13" spans="1:25" ht="30" x14ac:dyDescent="0.25">
@@ -1611,13 +1635,13 @@
         <v>131</v>
       </c>
       <c r="P13" s="4" t="s">
-        <v>190</v>
-      </c>
-      <c r="Q13" s="2" t="s">
-        <v>209</v>
+        <v>189</v>
+      </c>
+      <c r="Q13" s="4" t="s">
+        <v>208</v>
       </c>
       <c r="T13" s="2" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
     </row>
     <row r="14" spans="1:25" x14ac:dyDescent="0.25">
@@ -1643,7 +1667,13 @@
         <v>132</v>
       </c>
       <c r="P14" s="4" t="s">
-        <v>189</v>
+        <v>188</v>
+      </c>
+      <c r="Q14" s="4" t="s">
+        <v>203</v>
+      </c>
+      <c r="R14" s="7" t="s">
+        <v>210</v>
       </c>
     </row>
     <row r="15" spans="1:25" x14ac:dyDescent="0.25">
@@ -1669,7 +1699,13 @@
         <v>145</v>
       </c>
       <c r="P15" s="4" t="s">
-        <v>191</v>
+        <v>190</v>
+      </c>
+      <c r="Q15" s="7" t="s">
+        <v>207</v>
+      </c>
+      <c r="R15" s="7" t="s">
+        <v>211</v>
       </c>
     </row>
     <row r="16" spans="1:25" ht="30" x14ac:dyDescent="0.25">
@@ -1691,8 +1727,11 @@
       <c r="P16" s="4" t="s">
         <v>174</v>
       </c>
-    </row>
-    <row r="17" spans="1:17" ht="30" x14ac:dyDescent="0.25">
+      <c r="R16" s="4" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="17" spans="1:18" ht="30" x14ac:dyDescent="0.25">
       <c r="A17" s="2">
         <v>16</v>
       </c>
@@ -1711,8 +1750,11 @@
       <c r="P17" s="4" t="s">
         <v>176</v>
       </c>
-    </row>
-    <row r="18" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R17" s="4" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="18" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A18" s="2">
         <v>17</v>
       </c>
@@ -1731,11 +1773,11 @@
       <c r="P18" s="4" t="s">
         <v>165</v>
       </c>
-      <c r="Q18" s="4" t="s">
-        <v>204</v>
-      </c>
-    </row>
-    <row r="19" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R18" s="7" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="19" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A19" s="2">
         <v>18</v>
       </c>
@@ -1754,11 +1796,11 @@
       <c r="P19" s="7" t="s">
         <v>166</v>
       </c>
-      <c r="Q19" s="7" t="s">
-        <v>208</v>
-      </c>
-    </row>
-    <row r="20" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R19" s="4" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="20" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A20" s="2">
         <v>19</v>
       </c>
@@ -1778,7 +1820,7 @@
         <v>170</v>
       </c>
     </row>
-    <row r="21" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A21" s="2">
         <v>20</v>
       </c>
@@ -1792,7 +1834,7 @@
         <v>171</v>
       </c>
     </row>
-    <row r="22" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A22" s="2">
         <v>21</v>
       </c>
@@ -1806,7 +1848,7 @@
         <v>172</v>
       </c>
     </row>
-    <row r="23" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A23" s="2">
         <v>22</v>
       </c>
@@ -1820,7 +1862,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="24" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A24" s="2">
         <v>23</v>
       </c>
@@ -1834,7 +1876,7 @@
         <v>178</v>
       </c>
     </row>
-    <row r="25" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A25" s="2">
         <v>24</v>
       </c>
@@ -1848,7 +1890,7 @@
         <v>180</v>
       </c>
     </row>
-    <row r="26" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A26" s="2">
         <v>25</v>
       </c>
@@ -1859,7 +1901,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="27" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A27" s="2">
         <v>26</v>
       </c>
@@ -1867,7 +1909,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="28" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A28" s="2">
         <v>27</v>
       </c>
@@ -1875,7 +1917,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="29" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A29" s="2">
         <v>28</v>
       </c>
@@ -1883,7 +1925,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="30" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A30" s="2">
         <v>29</v>
       </c>
@@ -1891,7 +1933,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="31" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A31" s="2">
         <v>30</v>
       </c>
@@ -1899,7 +1941,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="32" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A32" s="2">
         <v>31</v>
       </c>

</xml_diff>

<commit_message>
update sgs and init VT5
</commit_message>
<xml_diff>
--- a/_other/WeekPlan.xlsx
+++ b/_other/WeekPlan.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Dev\exchange\RichLaughter\_other\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E6E93666-71D2-4FBD-8214-49FF36ADF10B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1CDA5158-F70A-4463-BDFC-9E89DC746DAE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="257" uniqueCount="255">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="265" uniqueCount="263">
   <si>
     <t>Новый тест с использованием БД</t>
   </si>
@@ -800,6 +800,30 @@
   </si>
   <si>
     <t>Провести child_test для потенциальных фьючерсов (SRU5,EDU5,GAZPF,SBERF,SVU5,VBU5,SF,NA)</t>
+  </si>
+  <si>
+    <t>Протестить BR и NG за 3 месяца</t>
+  </si>
+  <si>
+    <t>Какой-нибудь пробойный робот с adx и осцилятором с направлением тренда</t>
+  </si>
+  <si>
+    <t>STA4 (STA3 + adx + uo (или что-то другое) + работа в боковике (ggd или bb))</t>
+  </si>
+  <si>
+    <t>ranger + anger</t>
+  </si>
+  <si>
+    <t>Подумать над obbi</t>
+  </si>
+  <si>
+    <t>Подумать над новым индикатором выгоды</t>
+  </si>
+  <si>
+    <t>Revan на нестабильном тренде, кто-то другой на стабильном.</t>
+  </si>
+  <si>
+    <t>Стопнутый GGD (стоп можно по adx или альтернативе) Можно по линии в 2х спредов)</t>
   </si>
 </sst>
 </file>
@@ -863,7 +887,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.79998168889431442"/>
+        <fgColor theme="8" tint="0.59999389629810485"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1284,7 +1308,7 @@
         <v>45908</v>
       </c>
     </row>
-    <row r="2" spans="1:25" ht="60" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:25" ht="45" x14ac:dyDescent="0.25">
       <c r="A2" s="2">
         <v>1</v>
       </c>
@@ -1327,8 +1351,8 @@
       <c r="R2" s="4" t="s">
         <v>185</v>
       </c>
-      <c r="S2" s="13" t="s">
-        <v>254</v>
+      <c r="S2" s="4" t="s">
+        <v>253</v>
       </c>
       <c r="T2" s="2" t="s">
         <v>241</v>
@@ -1383,6 +1407,9 @@
       <c r="R3" s="4" t="s">
         <v>214</v>
       </c>
+      <c r="S3" s="13" t="s">
+        <v>254</v>
+      </c>
       <c r="T3" s="2" t="s">
         <v>240</v>
       </c>
@@ -1433,6 +1460,9 @@
       <c r="R4" s="4" t="s">
         <v>217</v>
       </c>
+      <c r="S4" s="13" t="s">
+        <v>248</v>
+      </c>
       <c r="T4" s="2" t="s">
         <v>252</v>
       </c>
@@ -1627,6 +1657,9 @@
       <c r="R8" s="4" t="s">
         <v>227</v>
       </c>
+      <c r="S8" s="2" t="s">
+        <v>255</v>
+      </c>
       <c r="T8" s="2" t="s">
         <v>247</v>
       </c>
@@ -1675,7 +1708,7 @@
         <v>225</v>
       </c>
       <c r="T9" s="2" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="U9" s="2" t="s">
         <v>228</v>
@@ -1722,7 +1755,7 @@
         <v>129</v>
       </c>
       <c r="T10" s="2" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="U10" s="2" t="s">
         <v>230</v>
@@ -1769,7 +1802,7 @@
         <v>245</v>
       </c>
       <c r="T11" s="2" t="s">
-        <v>250</v>
+        <v>256</v>
       </c>
       <c r="U11" s="2" t="s">
         <v>251</v>
@@ -1816,10 +1849,13 @@
         <v>239</v>
       </c>
       <c r="T12" s="2" t="s">
-        <v>253</v>
+        <v>257</v>
       </c>
       <c r="V12" s="2" t="s">
         <v>186</v>
+      </c>
+      <c r="W12" s="2" t="s">
+        <v>260</v>
       </c>
       <c r="X12" s="2" t="s">
         <v>175</v>
@@ -1856,6 +1892,9 @@
       <c r="R13" s="4" t="s">
         <v>244</v>
       </c>
+      <c r="T13" s="2" t="s">
+        <v>258</v>
+      </c>
     </row>
     <row r="14" spans="1:25" ht="30" x14ac:dyDescent="0.25">
       <c r="A14" s="2">
@@ -1888,8 +1927,11 @@
       <c r="R14" s="4" t="s">
         <v>243</v>
       </c>
-    </row>
-    <row r="15" spans="1:25" ht="30" x14ac:dyDescent="0.25">
+      <c r="T14" s="2" t="s">
+        <v>259</v>
+      </c>
+    </row>
+    <row r="15" spans="1:25" ht="45" x14ac:dyDescent="0.25">
       <c r="A15" s="2">
         <v>14</v>
       </c>
@@ -1920,8 +1962,11 @@
       <c r="R15" s="4" t="s">
         <v>226</v>
       </c>
-    </row>
-    <row r="16" spans="1:25" ht="30" x14ac:dyDescent="0.25">
+      <c r="T15" s="2" t="s">
+        <v>261</v>
+      </c>
+    </row>
+    <row r="16" spans="1:25" ht="60" x14ac:dyDescent="0.25">
       <c r="A16" s="2">
         <v>15</v>
       </c>
@@ -1942,6 +1987,9 @@
       </c>
       <c r="R16" s="4" t="s">
         <v>5</v>
+      </c>
+      <c r="T16" s="2" t="s">
+        <v>262</v>
       </c>
     </row>
     <row r="17" spans="1:18" ht="30" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Somebody ones told me...
</commit_message>
<xml_diff>
--- a/_other/WeekPlan.xlsx
+++ b/_other/WeekPlan.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Dev\exchange\RichLaughter\_other\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{22A7DC44-3086-4A6F-9D21-FF459F9AB117}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3DBAD27F-367D-4E6F-9DDE-8E78A629A75F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="303" uniqueCount="300">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="304" uniqueCount="301">
   <si>
     <t>Новый тест с использованием БД</t>
   </si>
@@ -862,9 +862,6 @@
     <t>Сделать аналоги PSTA6 на GGD вместо smas</t>
   </si>
   <si>
-    <t>Попробовать обновить оптуну на 2 фактора, прибыль и кол-во сделок</t>
-  </si>
-  <si>
     <t>PSTA7_DODO</t>
   </si>
   <si>
@@ -935,6 +932,12 @@
   </si>
   <si>
     <t>Стопнутый GGD (стоп можно по adx или альтернативе) Можно по линии в 2х спредов) Стоп можно по буфферу от последнего фрактала</t>
+  </si>
+  <si>
+    <t>PTA25_TASSADAR</t>
+  </si>
+  <si>
+    <t>Трейлинг-стоп</t>
   </si>
 </sst>
 </file>
@@ -1733,10 +1736,10 @@
         <v>251</v>
       </c>
       <c r="T2" s="4" t="s">
+        <v>283</v>
+      </c>
+      <c r="U2" s="2" t="s">
         <v>284</v>
-      </c>
-      <c r="U2" s="2" t="s">
-        <v>285</v>
       </c>
       <c r="V2" s="2" t="s">
         <v>240</v>
@@ -1795,13 +1798,13 @@
         <v>252</v>
       </c>
       <c r="T3" s="4" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="U3" s="2" t="s">
-        <v>283</v>
+        <v>288</v>
       </c>
       <c r="V3" s="2" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="W3" s="2" t="s">
         <v>196</v>
@@ -1854,9 +1857,6 @@
         <v>247</v>
       </c>
       <c r="T4" s="4" t="s">
-        <v>290</v>
-      </c>
-      <c r="U4" s="2" t="s">
         <v>289</v>
       </c>
       <c r="V4" s="2" t="s">
@@ -1910,10 +1910,10 @@
         <v>266</v>
       </c>
       <c r="T5" s="4" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="V5" s="2" t="s">
-        <v>245</v>
+        <v>229</v>
       </c>
       <c r="W5" s="2" t="s">
         <v>204</v>
@@ -1969,7 +1969,7 @@
         <v>194</v>
       </c>
       <c r="V6" s="2" t="s">
-        <v>229</v>
+        <v>246</v>
       </c>
       <c r="W6" s="2" t="s">
         <v>205</v>
@@ -2021,11 +2021,11 @@
       <c r="S7" s="4" t="s">
         <v>269</v>
       </c>
-      <c r="T7" s="2" t="s">
-        <v>287</v>
+      <c r="T7" s="4" t="s">
+        <v>245</v>
       </c>
       <c r="V7" s="2" t="s">
-        <v>246</v>
+        <v>253</v>
       </c>
       <c r="W7" s="2" t="s">
         <v>206</v>
@@ -2074,11 +2074,11 @@
       <c r="S8" s="12" t="s">
         <v>273</v>
       </c>
-      <c r="T8" s="2" t="s">
-        <v>288</v>
+      <c r="T8" s="14" t="s">
+        <v>286</v>
       </c>
       <c r="V8" s="2" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="W8" s="2" t="s">
         <v>218</v>
@@ -2127,8 +2127,11 @@
       <c r="S9" s="4" t="s">
         <v>274</v>
       </c>
+      <c r="T9" s="14" t="s">
+        <v>287</v>
+      </c>
       <c r="V9" s="2" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="W9" s="2" t="s">
         <v>228</v>
@@ -2177,9 +2180,11 @@
       <c r="S10" s="4" t="s">
         <v>259</v>
       </c>
-      <c r="T10" s="9"/>
+      <c r="T10" s="4" t="s">
+        <v>282</v>
+      </c>
       <c r="V10" s="2" t="s">
-        <v>255</v>
+        <v>258</v>
       </c>
       <c r="W10" s="2" t="s">
         <v>230</v>
@@ -2229,7 +2234,7 @@
         <v>260</v>
       </c>
       <c r="V11" s="2" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="W11" s="2" t="s">
         <v>250</v>
@@ -2244,7 +2249,7 @@
         <v>238</v>
       </c>
     </row>
-    <row r="12" spans="1:110" ht="45" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:110" ht="90" x14ac:dyDescent="0.25">
       <c r="A12" s="2">
         <v>11</v>
       </c>
@@ -2279,7 +2284,7 @@
         <v>262</v>
       </c>
       <c r="V12" s="2" t="s">
-        <v>257</v>
+        <v>298</v>
       </c>
       <c r="W12" s="2" t="s">
         <v>267</v>
@@ -2294,7 +2299,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="13" spans="1:110" ht="90" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:110" ht="30" x14ac:dyDescent="0.25">
       <c r="A13" s="2">
         <v>12</v>
       </c>
@@ -2329,10 +2334,13 @@
         <v>263</v>
       </c>
       <c r="V13" s="2" t="s">
-        <v>299</v>
+        <v>261</v>
       </c>
       <c r="W13" s="2" t="s">
         <v>268</v>
+      </c>
+      <c r="X13" s="2" t="s">
+        <v>300</v>
       </c>
       <c r="Y13" s="2" t="s">
         <v>248</v>
@@ -2373,10 +2381,10 @@
         <v>264</v>
       </c>
       <c r="T14" s="4" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="V14" s="2" t="s">
-        <v>261</v>
+        <v>271</v>
       </c>
       <c r="W14" s="2" t="s">
         <v>272</v>
@@ -2385,7 +2393,7 @@
         <v>249</v>
       </c>
     </row>
-    <row r="15" spans="1:110" ht="45" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:110" ht="30" x14ac:dyDescent="0.25">
       <c r="A15" s="2">
         <v>14</v>
       </c>
@@ -2420,13 +2428,10 @@
         <v>265</v>
       </c>
       <c r="T15" s="7" t="s">
-        <v>294</v>
-      </c>
-      <c r="V15" s="2" t="s">
-        <v>271</v>
+        <v>293</v>
       </c>
       <c r="W15" s="2" t="s">
-        <v>275</v>
+        <v>291</v>
       </c>
     </row>
     <row r="16" spans="1:110" ht="30" x14ac:dyDescent="0.25">
@@ -2452,13 +2457,10 @@
         <v>5</v>
       </c>
       <c r="S16" s="4" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="T16" s="7" t="s">
-        <v>295</v>
-      </c>
-      <c r="W16" s="2" t="s">
-        <v>292</v>
+        <v>294</v>
       </c>
     </row>
     <row r="17" spans="1:20" ht="30" x14ac:dyDescent="0.25">
@@ -2484,10 +2486,10 @@
         <v>210</v>
       </c>
       <c r="S17" s="7" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="T17" s="4" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
     </row>
     <row r="18" spans="1:20" x14ac:dyDescent="0.25">
@@ -2513,10 +2515,10 @@
         <v>211</v>
       </c>
       <c r="S18" s="7" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="T18" s="7" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
     </row>
     <row r="19" spans="1:20" x14ac:dyDescent="0.25">
@@ -2542,10 +2544,10 @@
         <v>212</v>
       </c>
       <c r="S19" s="7" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="T19" s="4" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
     </row>
     <row r="20" spans="1:20" x14ac:dyDescent="0.25">
@@ -2571,7 +2573,10 @@
         <v>213</v>
       </c>
       <c r="S20" s="7" t="s">
-        <v>280</v>
+        <v>279</v>
+      </c>
+      <c r="T20" s="4" t="s">
+        <v>299</v>
       </c>
     </row>
     <row r="21" spans="1:20" x14ac:dyDescent="0.25">
@@ -2591,7 +2596,7 @@
         <v>215</v>
       </c>
       <c r="S21" s="7" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
     </row>
     <row r="22" spans="1:20" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
prepare test for cryptos 30min
</commit_message>
<xml_diff>
--- a/_other/WeekPlan.xlsx
+++ b/_other/WeekPlan.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Dev\exchange\RichLaughter\_other\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EF16A015-89F4-490D-897A-85081BED06D5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{47C12082-73F2-41B3-8C21-169C40788B34}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Лист1" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="318" uniqueCount="315">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="319" uniqueCount="316">
   <si>
     <t>Новый тест с использованием БД</t>
   </si>
@@ -980,6 +980,9 @@
   </si>
   <si>
     <t>Провести оптимизацию под 30m для Bitget и Bybit</t>
+  </si>
+  <si>
+    <t>Удалить данные 17.09 по фьючам с ошибочной 3-4 процентной сделкой</t>
   </si>
 </sst>
 </file>
@@ -1820,6 +1823,9 @@
         <v>301</v>
       </c>
       <c r="Z2" s="2" t="s">
+        <v>314</v>
+      </c>
+      <c r="AA2" s="2" t="s">
         <v>305</v>
       </c>
       <c r="AB2" s="13" t="s">
@@ -1884,10 +1890,10 @@
       <c r="U3" s="4" t="s">
         <v>298</v>
       </c>
-      <c r="Y3" s="2" t="s">
-        <v>314</v>
-      </c>
       <c r="Z3" s="2" t="s">
+        <v>315</v>
+      </c>
+      <c r="AA3" s="2" t="s">
         <v>306</v>
       </c>
       <c r="AB3" s="14" t="s">
@@ -1949,7 +1955,7 @@
       <c r="U4" s="7" t="s">
         <v>299</v>
       </c>
-      <c r="Z4" s="2" t="s">
+      <c r="AA4" s="2" t="s">
         <v>307</v>
       </c>
       <c r="AB4" s="13" t="s">
@@ -2005,7 +2011,7 @@
       <c r="T5" s="4" t="s">
         <v>286</v>
       </c>
-      <c r="Z5" s="2" t="s">
+      <c r="AA5" s="2" t="s">
         <v>308</v>
       </c>
       <c r="AB5" s="14" t="s">
@@ -2064,7 +2070,7 @@
       <c r="T6" s="4" t="s">
         <v>193</v>
       </c>
-      <c r="Z6" s="2" t="s">
+      <c r="AA6" s="2" t="s">
         <v>309</v>
       </c>
       <c r="AB6" s="14" t="s">
@@ -2123,7 +2129,7 @@
       <c r="T7" s="4" t="s">
         <v>244</v>
       </c>
-      <c r="Z7" s="2" t="s">
+      <c r="AA7" s="2" t="s">
         <v>310</v>
       </c>
       <c r="AB7" s="14" t="s">
@@ -2179,7 +2185,7 @@
       <c r="T8" s="4" t="s">
         <v>283</v>
       </c>
-      <c r="Z8" s="2" t="s">
+      <c r="AA8" s="2" t="s">
         <v>311</v>
       </c>
       <c r="AB8" s="14" t="s">
@@ -2235,7 +2241,7 @@
       <c r="T9" s="4" t="s">
         <v>284</v>
       </c>
-      <c r="Z9" s="2" t="s">
+      <c r="AA9" s="2" t="s">
         <v>312</v>
       </c>
       <c r="AB9" s="13" t="s">
@@ -2291,7 +2297,7 @@
       <c r="T10" s="4" t="s">
         <v>279</v>
       </c>
-      <c r="Z10" s="2" t="s">
+      <c r="AA10" s="2" t="s">
         <v>313</v>
       </c>
       <c r="AB10" s="15" t="s">

</xml_diff>